<commit_message>
v15: bandejas demo completas para los ocho cargos, espejadas en historia y bases
- Director: medición postural pendiente de aceptar (DEM-003) y su
  coordinación En ajuste esperando a la dirección.
- Gestor de Datos 1: «Tablero BI de control · fase 2» pendiente.
- Supervisor: «Cápsulas de seguridad para líderes de línea» pendientes,
  120 personas a impactar y hoja de vida de contenidos definida.
- Dirección (CEO/Gerente): 2 casos por resolver (producto+coordinación).
- Bases de alimentación con filas espejo (segundo diseño, cápsulas de
  refuerzo 80 personas; BI ya traía la fase 2 pendiente).
- Historia de usuario actualizada con los casos demo concretos.
- Capturas de la guía refrescadas; 16 verificaciones en verde y la
  carga de Base_BI alimenta la bandeja de GD1.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J7RCgg76gjh3iFAK7tfLBo
</commit_message>
<xml_diff>
--- a/entregables/gestion-proyectos/Historia_de_usuario_Rehavid_v15.xlsx
+++ b/entregables/gestion-proyectos/Historia_de_usuario_Rehavid_v15.xlsx
@@ -4635,7 +4635,7 @@
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>Abra Mi trabajo con su sesión: la sección «Para resolver como dirección» lista los ajustes de todos los cargos (en la base demostrativa, el Tablero BI de DEM-001). Use «Resolver ajuste» y pruebe las cuatro decisiones.</t>
+          <t>Abra Mi trabajo con su sesión: la sección «Para resolver como dirección» lista los ajustes de todos los cargos (en la demo: el Tablero BI de DEM-001 y la coordinación de DEM-003). Use «Resolver ajuste» y pruebe las cuatro decisiones.</t>
         </is>
       </c>
       <c r="E14" s="10" t="inlineStr">
@@ -5127,7 +5127,7 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Su Mi trabajo trae la sección «Para resolver como dirección» con los ajustes de todos los cargos. Resuelva el del Tablero BI demostrativo con contrapropuesta; observe el estado que queda.</t>
+          <t>Su Mi trabajo trae la sección «Para resolver como dirección» con dos casos demo: el Tablero BI de DEM-001 y la coordinación de DEM-003. Resuelva uno con contrapropuesta; observe el estado que queda.</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -5498,17 +5498,17 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Recibir la coordinación Tipo 2 en Mi trabajo</t>
+          <t>Revisar sus coordinaciones Tipo 2 en Mi trabajo</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Active un Tipo 2 y abra Mi trabajo.</t>
+          <t>Abra Mi trabajo: la demo trae la coordinación de DEM-001 (aceptada) y la de DEM-003 «En ajuste» con la propuesta que usted mismo hizo por el corrimiento de la parada de mantenimiento.</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>La coordinación llega como tarjeta independiente con su ciclo propio (validado en la segunda ronda; confirme que sigue igual tras la simplificación).</t>
+          <t>Cada coordinación es una tarjeta independiente con su ciclo y su historial; la que está en ajuste espera la decisión de la dirección.</t>
         </is>
       </c>
       <c r="F11" s="19" t="n"/>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>Acepte la asignación de mediciones declarando tiempo y capacidad; en otro producto proponga ajuste.</t>
+          <t>Acepte la «Medición objetiva de carga postural» (DEM-003) que llega pendiente en su bandeja, declarando tiempo y capacidad; en otro producto proponga ajuste.</t>
         </is>
       </c>
       <c r="E12" s="10" t="inlineStr">
@@ -6569,17 +6569,17 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Revisar la asignación de cápsulas</t>
+          <t>Revisar sus asignaciones de cápsulas</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>En Mi trabajo revise su tarjeta de cápsulas.</t>
+          <t>En Mi trabajo revise sus dos tarjetas demo: las cápsulas en curso (DEM-001) y las «Cápsulas de seguridad para líderes de línea» (DEM-002) pendientes, con 120 personas a impactar y su hoja de vida de contenidos definida.</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>Muestra horas vendidas y personas a impactar; los botones de aceptar aparecen en la propia tarjeta cuando está pendiente (su N°3: verifique que ahora es visible).</t>
+          <t>Los botones «Aceptar asignación» y «Proponer ajuste» están en la propia tarjeta pendiente (su N°3 de la segunda ronda: verifique que ahora es visible).</t>
         </is>
       </c>
       <c r="F13" s="19" t="n"/>
@@ -6603,7 +6603,7 @@
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>Acepte declarando tiempo y capacidad; en otra asignación proponga ajuste por disponibilidad de producción.</t>
+          <t>Acepte las cápsulas pendientes declarando tiempo y capacidad; luego proponga un ajuste por disponibilidad de producción.</t>
         </is>
       </c>
       <c r="E14" s="10" t="inlineStr">
@@ -7042,7 +7042,7 @@
       </c>
       <c r="E12" s="10" t="inlineStr">
         <is>
-          <t>El resumen (Pendientes · En ajuste · Aceptadas · Coordinación) encabeza su bandeja; su producto aparece con las alertas dentro de la tarjeta.</t>
+          <t>Su bandeja demo trae el «Tablero BI de control · fase 2» (DEM-003) pendiente de aceptar y el tablero de DEM-001 en ajuste esperando a la dirección, con las alertas dentro de cada tarjeta.</t>
         </is>
       </c>
       <c r="F12" s="19" t="n"/>
@@ -7066,7 +7066,7 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Acepte la asignación del tablero; en otra pruebe proponer ajuste y reciba la decisión de la dirección.</t>
+          <t>Acepte la fase 2 declarando tiempo y capacidad; observe en la otra tarjeta la negociación en curso.</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">

</xml_diff>